<commit_message>
Add login column to employees for Access Graph persona setup
Platform logins (surname, lowercase, matching the existing email
local-part convention) for all 6 employees -- needed so the Scenario 2
role setup can bind Access Graph personas to actual usernames instead
of just role labels. Deliberately left out of data_sensitivity_catalog:
masking a login would break the very access-policy binding it exists
to support. Regenerated the xlsx export from a fresh init.sql run to
keep it in sync.
</commit_message>
<xml_diff>
--- a/docs/demo-retail/database/torgline-demo-data.xlsx
+++ b/docs/demo-retail/database/torgline-demo-data.xlsx
@@ -1770,7 +1770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1780,6 +1780,7 @@
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1825,6 +1826,11 @@
           <t>email</t>
         </is>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1858,6 +1864,11 @@
           <t>p.sokolov@torgline-demo.ru</t>
         </is>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>sokolov</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1889,6 +1900,11 @@
       <c r="G5" s="3" t="inlineStr">
         <is>
           <t>n.dmitrieva@torgline-demo.ru</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>dmitrieva</t>
         </is>
       </c>
     </row>
@@ -1920,6 +1936,11 @@
           <t>k.egorov@torgline-demo.ru</t>
         </is>
       </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>egorov</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1949,6 +1970,11 @@
           <t>a.smirnova@torgline-demo.ru</t>
         </is>
       </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>smirnova</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1978,6 +2004,11 @@
           <t>e.voloshina@torgline-demo.ru</t>
         </is>
       </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>voloshina</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -2007,10 +2038,15 @@
           <t>e.petrova@torgline-demo.ru</t>
         </is>
       </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>petrova</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Turn sensitivity categories into real, queryable data
pii/financial/contract_terms were only explained in a SQL comment,
invisible to anyone reading the table itself. Added sensitivity_levels
(description + masking guidance per category) and made
data_sensitivity_catalog.sensitivity a real FK into it, so the meaning
is enforced and joinable, not just documented in the script's source.
Re-verified init.sql end-to-end and regenerated the xlsx export
(now 17 sheets) to match.
</commit_message>
<xml_diff>
--- a/docs/demo-retail/database/torgline-demo-data.xlsx
+++ b/docs/demo-retail/database/torgline-demo-data.xlsx
@@ -22,7 +22,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="loyalty_transactions" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="supplier_claims" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="employees" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_sensitivity_catalog" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sensitivity_levels" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_sensitivity_catalog" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2058,6 +2059,103 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>sensitivity_levels — Описание категорий чувствительности</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>sensitivity_code</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>masking_guidance</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>pii</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Персональные данные — прямо идентифицируют конкретного человека: ФИО, телефон, e-mail, номер карты лояльности, юридический адрес.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Маскировать для любой роли, которой не нужно знать личность конкретного человека для выполнения задачи (например, специалист поддержки видит историю покупок, но не полный номер карты). Кандидат на контекстный BERT-фильтр — распознавание по типу сущности (ФИО/телефон/e-mail), а не по конкретному списку значений.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>financial</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Финансовые и регистрационные данные компании — банковские реквизиты, ИНН/КПП/ОГРН, закупочные цены, себестоимость, маржа.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Маскировать для ролей без доступа к финансовым показателям (например, «директор магазина» видит выручку своего магазина, но не закупочную стоимость и маржу — см. Сценарий 2). Для банковских реквизитов поставщика — видно только ролям, ответственным за оплату.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>contract_terms</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Содержательные условия договора, а не отдельный персональный/финансовый атрибут — например, весь раздел «Гарантийные обязательства».</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Маскировать целиком по явному, настроенному правилу (не по regex общего назначения, который совпадает по формату числа/даты) — раздел скрывается независимо от конкретной формулировки. См. демо-Сценарий 9: тест «жёсткое / мягкое маскирование» именно на этом типе данных, потому что ошибочно скрытое условие меняет правовой смысл ответа, а не просто прячет цифру.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>